<commit_message>
Add election_data and agenda_implementation datasets; finalise commission_formation for release
- election_data: euandi 2024 VAA coding (Ireland + EU-level), pipeline, docs,
  figures, tests. party_id "Greens" renamed to "EGP" for acronym consistency.
- agenda_implementation: Phase 1 (Annex IV status, term corpus, spine), docs,
  figures, tests.
- commission_formation: re-parsed Annex I (127 WP items), LLM-classified
  mission-letter commitments (1057, cache shipped), CODEBOOK clarifies
  type_of_act nulls for Annexes II/III.
- Site: data.qmd sections for all three datasets; full quarto render in docs/.
- Metadata: CITATION.cff and .zenodo.json cover all three datasets.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datasets/commission_formation/data/output/work_programme_items.xlsx
+++ b/datasets/commission_formation/data/output/work_programme_items.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H114"/>
+  <dimension ref="A1:H128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,18 +483,30 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>11.</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Competitiveness and Decarbonisation</t>
+          <t>Competitiveness Compass</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Competitiveness</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -509,18 +521,30 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>12.</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Single Market Strategy</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Competitiveness</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -535,18 +559,30 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>13.</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Innovation</t>
+          <t>First Omnibus package on sustainability</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Simplification</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -561,18 +597,30 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>14.</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Innovation</t>
+          <t>Second Omnibus package on investment simplification</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Simplification</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -587,18 +635,30 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15.</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Innovation</t>
+          <t>Third Omnibus package, including on small mid-caps and removal of paper requirements</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Simplification</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -613,18 +673,30 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>16.</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Competitiveness</t>
+          <t>Digital package</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Simplification</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -639,18 +711,30 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17.</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Competitiveness and Decarbonisation</t>
+          <t>European Business Wallet</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Simplification</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -665,18 +749,30 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>18.</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Simplification</t>
+          <t>Clean Industrial Deal</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Competitiveness and Decarbonisation</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -691,18 +787,30 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>19.</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Action plan on affordable energy</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Competitiveness and Decarbonisation</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -717,18 +825,30 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>20.</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>Industrial Decarbonisation Accelerator Act</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>Competitiveness and Decarbonisation</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -743,18 +863,30 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>21.</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>EU Start-up and Scale-up Strategy</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Competitiveness and Decarbonisation</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -769,18 +901,30 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>22.</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Preparedness and Resilience</t>
+          <t>Communication on a Savings and Investments Union</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Competitiveness</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -795,18 +939,30 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23.</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Preparedness and Resilience</t>
+          <t>Review of the Securitisation Framework</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Competitiveness</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -821,18 +977,30 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>24.</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Digital Networks Act</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -847,18 +1015,30 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>25.</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>AI Continent Action Plan</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -873,18 +1053,30 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>26.</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Quantum Strategy of EU</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -899,18 +1091,30 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>27.</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>EU Space Act</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Competitiveness</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -925,18 +1129,30 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>28.</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Bioeconomy Strategy</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Competitiveness and Decarbonisation</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Non-legislative or legislative</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -951,18 +1167,30 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>29.</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Social fairness</t>
+          <t>Targeted revision of the REACH Regulation</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Simplification</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -977,18 +1205,30 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>30.</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Social fairness</t>
+          <t>Roadmap towards ending Russian energy imports</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1003,18 +1243,30 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>31.</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Competitiveness</t>
+          <t>Sustainable Transport Investment Plan</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Competitiveness and Decarbonisation A new era for European Defence and Security</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Q3 2025</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1029,18 +1281,30 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>32.</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Social fairness</t>
+          <t>White Paper on the Future of European Defence</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1055,18 +1319,30 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>33.</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Decarbonisation</t>
+          <t>EU Preparedness Union Strategy</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Preparedness and Resilience</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1081,18 +1357,30 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>34.</t>
+          <t>23</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Competitiveness and Decarbonisation</t>
+          <t>Critical Medicines Act</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Preparedness and Resilience</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1107,18 +1395,30 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>35.</t>
+          <t>23</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Simplification</t>
+          <t>Strategy to support medical countermeasures against public health threats</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Preparedness and Resilience</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1133,18 +1433,30 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>36.</t>
+          <t>23</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Competitiveness</t>
+          <t>EU Stockpiling Strategy</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Preparedness and Resilience</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1159,18 +1471,30 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>37.</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Preparedness and Resilience</t>
+          <t>New European Internal Security Strategy</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1185,18 +1509,30 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>38.</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Democracy</t>
+          <t>New rules on drug precursors</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1211,18 +1547,30 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>39.</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Equality</t>
+          <t>Firearms Trafficking Directive</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1237,18 +1585,30 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>40.</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Equality</t>
+          <t>Action plan on the cybersecurity of hospitals and healthcare providers</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1263,18 +1623,30 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>41.</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Geopolitics</t>
+          <t>New common approach on returns</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1289,18 +1661,30 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>42.</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Geopolitics</t>
+          <t>European Migration and Asylum Strategy</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1315,18 +1699,30 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>43.</t>
+          <t>29</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Geopolitics</t>
+          <t>A new action plan to implement the European Pillar of Social Rights</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Social fairness</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1341,18 +1737,30 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>44.</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Future priority</t>
+          <t>Quality jobs roadmap</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Social fairness</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1367,18 +1775,30 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>45.</t>
+          <t>31</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Future priority</t>
+          <t>Union of Skills</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Competitiveness</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1388,27 +1808,35 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1.</t>
+          <t>32</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>2030 Consumer Agenda, including an action plan for consumers in the Single Market</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Fitness check on the legislative acquis in the digital policy area</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+          <t>Social fairness Sustaining our quality of life: food security, water and nature</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1418,27 +1846,35 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2.</t>
+          <t>33</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Q2 2025</t>
+          <t>European Climate Law amendment</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Fitness check on energy security architecture</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
+          <t>Decarbonisation</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1448,27 +1884,35 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>3.</t>
+          <t>34</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Q2 / Q3 2025</t>
+          <t>Vision for Agriculture and Food</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Fitness check on market access in inland waterway transport</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+          <t>Competitiveness and Decarbonisation</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1478,27 +1922,35 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>4.</t>
+          <t>35</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>Common Agricultural Policy simplification package</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Fitness Check of EU airports legislation</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
+          <t>Simplification</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1508,27 +1960,35 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>5.</t>
+          <t>36</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Q3 2025</t>
+          <t>Ocean Pact</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Evaluation of the Public Procurement Directives</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
+          <t>Competitiveness</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1538,27 +1998,35 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>6.</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>European Water Resilience Strategy</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Evaluation of EU rules on medical devices and in vitro diagnostics</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+          <t>Preparedness and Resilience Protecting our democracy, upholding our values</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1568,27 +2036,35 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>7.</t>
+          <t>38</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>European Democracy Shield</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Evaluation of the National Emission Reduction Commitments Directive</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
+          <t>Democracy</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Q3 2025</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1598,27 +2074,35 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>8.</t>
+          <t>38</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>EU Strategy to support, protect and empower the civil society</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Evaluation of radioactive waste directives</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+          <t>Democracy</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Q3 2025</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1628,27 +2112,35 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>9.</t>
+          <t>39</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>Roadmap for Women’s Rights</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Evaluation of the Pressure Equipment Directive and the Simple Pressure Vessels Directive</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
+          <t>Equality</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1658,27 +2150,35 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10.</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Q2 2025</t>
+          <t>New equality strategies for LGBTIQ</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Evaluation of the EU Lifts Directive</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+          <t>Equality A global Europe: Leveraging our power and partnerships</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1688,27 +2188,35 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>11.</t>
+          <t>41</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Q3 2025</t>
+          <t>Pact for the Mediterranean</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Evaluation of the Directive on Unfair trading practices in the agricultural and food supply chain</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+          <t>Geopolitics</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Q3 2025</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1718,27 +2226,35 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>12.</t>
+          <t>42</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>EU strategic approach to the Black Sea/ Black Sea Strategy</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Evaluation on the Land use, land-use change and forestry (LULUCF) Regulation</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
+          <t>Geopolitics</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1748,27 +2264,35 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>13.</t>
+          <t>43</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Q1/Q2 2025</t>
+          <t>Joint Communication on a new Strategic EU-India Agenda</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Evaluation of the Fishing Vessel Safety Directive</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
+          <t>Geopolitics Delivering together and preparing our Union for the future</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Non-legislative</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1778,27 +2302,35 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>14.</t>
+          <t>44</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>Post-2027 Multiannual Financial Framework proposals</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Evaluation of the Geo-blocking Regulation (GBR)</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
+          <t>Future priority</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Legislative</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Q3 2025</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1813,7 +2345,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>15.</t>
+          <t>1.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1824,7 +2356,7 @@
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Evaluation of State aid rules for banks in difficulties</t>
+          <t>Fitness check on the legislative acquis in the digital policy area</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
@@ -1843,18 +2375,18 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>16.</t>
+          <t>2.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Q3 2025</t>
+          <t>Q2 2025</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Evaluation of the Guarantee Notice</t>
+          <t>Fitness check on energy security architecture</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
@@ -1873,18 +2405,18 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>17.</t>
+          <t>3.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>Q2 / Q3 2025</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Evaluation of the Anti-tax Avoidance Directive (ATAD)</t>
+          <t>Fitness check on market access in inland waterway transport</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -1903,7 +2435,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>18.</t>
+          <t>4.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1914,7 +2446,7 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Evaluation of EU Rules of Origin</t>
+          <t>Fitness Check of EU airports legislation</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
@@ -1933,18 +2465,18 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>19.</t>
+          <t>5.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>Q3 2025</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Evaluation of the Defence Transfers Directive</t>
+          <t>Evaluation of the Public Procurement Directives</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
@@ -1963,7 +2495,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>20.</t>
+          <t>6.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1974,7 +2506,7 @@
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Evaluation of the Firearms Directive</t>
+          <t>Evaluation of EU rules on medical devices and in vitro diagnostics</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
@@ -1993,7 +2525,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>21.</t>
+          <t>7.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2004,7 +2536,7 @@
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Evaluation on the Innovation Fund</t>
+          <t>Evaluation of the National Emission Reduction Commitments Directive</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
@@ -2023,7 +2555,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>22.</t>
+          <t>8.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2034,7 +2566,7 @@
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Evaluation on the Modernisation Fund</t>
+          <t>Evaluation of radioactive waste directives</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
@@ -2053,18 +2585,18 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>23.</t>
+          <t>9.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Q3 2025</t>
+          <t>Q4 2025</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Evaluation of Regulation (EU) 2016/796 of EU Agency for Railways</t>
+          <t>Evaluation of the Pressure Equipment Directive and the Simple Pressure Vessels Directive</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
@@ -2083,18 +2615,18 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>24.</t>
+          <t>10.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Q3/Q4 2025</t>
+          <t>Q2 2025</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Ex-post evaluation of Connecting Europe Facility (CEF) 2014-2020</t>
+          <t>Evaluation of the EU Lifts Directive</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
@@ -2113,18 +2645,18 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>25.</t>
+          <t>11.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Q2 2025</t>
+          <t>Q3 2025</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Ex-post evaluation of Asylum, Migration, and Integration Fund (AMIF) 2014-2020</t>
+          <t>Evaluation of the Directive on Unfair trading practices in the agricultural and food supply chain</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
@@ -2143,18 +2675,18 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>26.</t>
+          <t>12.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Q2 2025</t>
+          <t>Q4 2025</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Ex-post evaluation of the Internal Security Fund – Borders and Visa (ISF-BV) 2014-2020</t>
+          <t>Evaluation on the Land use, land-use change and forestry (LULUCF) Regulation</t>
         </is>
       </c>
       <c r="G62" t="inlineStr"/>
@@ -2173,18 +2705,18 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>27.</t>
+          <t>13.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Q2 2025</t>
+          <t>Q1/Q2 2025</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Ex-post evaluation of the Internal Security Fund – Police (ISF-P) 2014-2020</t>
+          <t>Evaluation of the Fishing Vessel Safety Directive</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
@@ -2203,18 +2735,18 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>28.</t>
+          <t>14.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Q2 2025</t>
+          <t>Q4 2025</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Ex-post evaluation of the European Regional Development Fund and the Cohesion Fund 2014-2020</t>
+          <t>Evaluation of the Geo-blocking Regulation (GBR)</t>
         </is>
       </c>
       <c r="G64" t="inlineStr"/>
@@ -2233,18 +2765,18 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>29.</t>
+          <t>15.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Q2 2025</t>
+          <t>Q4 2025</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Ex post evaluation of the Fund for European Aid to the Most Deprived (FEAD) 2014-2020</t>
+          <t>Evaluation of State aid rules for banks in difficulties</t>
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
@@ -2263,7 +2795,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>30.</t>
+          <t>16.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2274,7 +2806,7 @@
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Ex post evaluation of European Social Fund and Youth Employment Initiative 2014-2020</t>
+          <t>Evaluation of the Guarantee Notice</t>
         </is>
       </c>
       <c r="G66" t="inlineStr"/>
@@ -2293,18 +2825,18 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>31.</t>
+          <t>17.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Q1-Q2 2025</t>
+          <t>Q4 2025</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Interim Evaluation of the European Defence Fund</t>
+          <t>Evaluation of the Anti-tax Avoidance Directive (ATAD)</t>
         </is>
       </c>
       <c r="G67" t="inlineStr"/>
@@ -2323,18 +2855,18 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>32.</t>
+          <t>18.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Q3 2025</t>
+          <t>Q4 2025</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Interim evaluation of the Customs 2021-2027 programme</t>
+          <t>Evaluation of EU Rules of Origin</t>
         </is>
       </c>
       <c r="G68" t="inlineStr"/>
@@ -2353,18 +2885,18 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>33.</t>
+          <t>19.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Q2 2025</t>
+          <t>Q4 2025</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Interim evaluation of the Customs Control Equipment Instrument (CCEI) programme</t>
+          <t>Evaluation of the Defence Transfers Directive</t>
         </is>
       </c>
       <c r="G69" t="inlineStr"/>
@@ -2383,7 +2915,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>34.</t>
+          <t>20.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2394,7 +2926,7 @@
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Interim Evaluation of the Fiscalis 2021-2027 programme</t>
+          <t>Evaluation of the Firearms Directive</t>
         </is>
       </c>
       <c r="G70" t="inlineStr"/>
@@ -2408,26 +2940,26 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>35.</t>
+          <t>21.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Interim evaluation of the Horizon Europe framework programme for Research and Innovation</t>
+          <t>Q4 2025</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>Q2 2025</t>
-        </is>
-      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Evaluation on the Innovation Fund</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
@@ -2438,26 +2970,26 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>36.</t>
+          <t>22.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Mid-term evaluation of the European Regional Development Fund, the Cohesion Fund and the Just Transition Fund 2021-2027</t>
+          <t>Q4 2025</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>Q2 2025</t>
-        </is>
-      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Evaluation on the Modernisation Fund</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
@@ -2468,26 +3000,26 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>37.</t>
+          <t>23.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Mid-term evaluation of the European Social Fund Plus 2021-2027</t>
+          <t>Q3 2025</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>Q2 2025</t>
-        </is>
-      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Evaluation of Regulation (EU) 2016/796 of EU Agency for Railways</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
@@ -2498,35 +3030,27 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>24.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>COM(2011)714 final Proposal for a COUNCIL DIRECTIVE on a common system of taxation Obsolete – the scope of the proposal has been partly</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>2011/0314 (CNS) applicable to interest and royalty payments made between associated companies taken over by the Directive implementing the OECD of different Member States Pillar 2 on minimum corporate taxation. The remaining issues the proposal intended to tackle will be addressed via an upcoming Omnibus act as a part of the simplification process.</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>DIRECTIVE</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
-      </c>
+          <t>Q3/Q4 2025</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Ex-post evaluation of Connecting Europe Facility (CEF) 2014-2020</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2536,35 +3060,27 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>25.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>COM(2011)827 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF Obsolete – the proposal is by now obsolete. The</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>2011/0391 (COD) THE COUNCIL on common rules for the allocation of slots at European Union Commission has launched a fitness-check and will airports decide on the basis of its findings on the way forward.</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>REGULATION</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
-      </c>
+          <t>Q2 2025</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Ex-post evaluation of Asylum, Migration, and Integration Fund (AMIF) 2014-2020</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2574,35 +3090,27 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>26.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>COM(2012)336 final Proposal for a COUNCIL REGULATION establishing a facility for providing Obsolete – the proposal needs to be updated as regards</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>2012/0164 (APP) financial assistance for Member States whose currency is not the euro i.a. the funding modalities of the Balance of Payments Facility and to integrate the lessons to be drawn from the recent crises, as well as the institutional, economic and financial sector developments since 2009, and their possible implication for the design and implementation of the facility, in line with the Council Conclusions of 27 March 2024.</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>REGULATION</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
-      </c>
+          <t>Q2 2025</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Ex-post evaluation of the Internal Security Fund – Borders and Visa (ISF-BV) 2014-2020</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2612,35 +3120,27 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>27.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>COM(2015)603 final Proposal for a COUNCIL DECISION laying down measures in view of No foreseeable agreement – in the context of the</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>2015/0250 (NLE) progressively establishing unified representation of the euro area in the discussions on Europe’s economic and financial International Monetary Fund sovereignty, the Commission will assess whether another proposal should be tabled or another type of approach should be chosen. 2 This list includes pending legislative proposals, which the Commission intends to withdraw within six months 22 No. References Title Reasons for withdrawal</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>DECISION</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
-      </c>
+          <t>Q2 2025</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Ex-post evaluation of the Internal Security Fund – Police (ISF-P) 2014-2020</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2650,35 +3150,27 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>28.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>COM(2017)276 final Proposal for a COUNCIL DIRECTIVE amending Directive 1999/62/EC on the No foreseeable agreement – the proposal is blocked with</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>2017/0115 (CNS) charging of heavy goods vehicles for the use of certain infrastructures, as regards no perspective of agreement. certain provisions on vehicle taxation</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>DIRECTIVE</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
+          <t>Q2 2025</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Ex-post evaluation of the European Regional Development Fund and the Cohesion Fund 2014-2020</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2688,35 +3180,27 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>29.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>COM(2017)647 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – the proposal has not been</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>2017/0288 (COD) THE COUNCIL amending Regulation (EC) No 1073/2009 on common rules for taken up for discussion in the Council and is by now access to the international market for coach and bus services outdated.</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>REGULATION</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
+          <t>Q2 2025</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Ex post evaluation of the Fund for European Aid to the Most Deprived (FEAD) 2014-2020</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2726,35 +3210,27 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>30.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>COM(2017)827 final Proposal for a COUNCIL REGULATION on the establishment of the European No foreseeable agreement - many of the changes</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>2017/0333 (APP) Monetary Fund proposed under this initiative have been incorporated into a separate revision of the European Stability Mechanism Treaty.</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>REGULATION</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
+          <t>Q3 2025</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Ex post evaluation of European Social Fund and Youth Employment Initiative 2014-2020</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2764,35 +3240,27 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>31.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>COM(2018)135 final Proposal for a DIRECTIVE OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – the proposal is blocked and</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>2018/0063B (COD) THE COUNCIL on credit servicers, credit purchasers and the recovery of further progress is unlikely. collateral</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>DIRECTIVE</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
+          <t>Q1-Q2 2025</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Interim Evaluation of the European Defence Fund</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2802,35 +3270,27 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>32.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>COM(2018)329 final Proposal for a COUNCIL DIRECTIVE amending Directive 2006/112/EC as No foreseeable agreement – discussions are suspended</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>2018/0164(CNS) regards the introduction of the detailed technical measures for the operation of since 2019 and further progress is unlikely. the definitive VAT system for the taxation of trade between Member States</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>DIRECTIVE</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
+          <t>Q3 2025</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Interim evaluation of the Customs 2021-2027 programme</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2840,35 +3300,27 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>33.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>COM(2018)339 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – the proposal is blocked and</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>2018/0171 (COD) THE COUNCIL on sovereign bond-backed securities further progress is unlikely.</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>REGULATION</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
+          <t>Q2 2025</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Interim evaluation of the Customs Control Equipment Instrument (CCEI) programme</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2878,35 +3330,27 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>34.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>COM(2018)387 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement - The proposal is outdated</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>2018/0212 (COD) THE COUNCIL on the establishment of a European Investment Stabilisation with the entry into force of NGEU and the Recovery and Function Resilience Facility (RRF) and the withdrawal of the so- called Budgetary Instrument for Convergence and Competitiveness (BICC) in February 2021.</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>REGULATION</t>
-        </is>
-      </c>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
+          <t>Q4 2025</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Interim Evaluation of the Fiscalis 2021-2027 programme</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2916,33 +3360,25 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>III</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>35.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>COM(2019)38 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF Obsolete – changes contained in this proposal have been</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>2019/0017 (COD) THE COUNCIL amending Regulation (EU) 2015/757 in order to take incorporated into the most recent EU ETS revision, appropriate account of the global data collection system for ship fuel oil adopted in 2023. consumption data</t>
-        </is>
-      </c>
+          <t>Interim evaluation of the Horizon Europe framework programme for Research and Innovation</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>REGULATION</t>
-        </is>
-      </c>
+      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>Q2 2025</t>
         </is>
       </c>
     </row>
@@ -2954,33 +3390,25 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>III</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>36.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>COM(2020)49 final Proposal for a COUNCIL DIRECTIVE on administrative cooperation in the field Obsolete - since the adoption of this proposal in 2020, a</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>2020/0022 (CNS) of taxation (codification) number of significant amendments have been adopted, making this codification proposal obsolete. The Commission will propose a new codified proposal. 23 No. References Title Reasons for withdrawal</t>
-        </is>
-      </c>
+          <t>Mid-term evaluation of the European Regional Development Fund, the Cohesion Fund and the Just Transition Fund 2021-2027</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>DIRECTIVE</t>
-        </is>
-      </c>
+      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>Q2 2025</t>
         </is>
       </c>
     </row>
@@ -2992,33 +3420,25 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>III</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>37.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>COM(2020)577 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF Obsolete – changes contained in this proposal have been</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>2020/0264 (COD) THE COUNCIL amending Regulation (EU) 2018/1139 as regards the capacity incorporated into the Single European Sky ("SES II +") of the European Union Aviation Safety Agency to act as Performance Review Regulation. Body of the Single European Sky</t>
-        </is>
-      </c>
+          <t>Mid-term evaluation of the European Social Fund Plus 2021-2027</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>REGULATION</t>
-        </is>
-      </c>
+      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>Q2 2025</t>
         </is>
       </c>
     </row>
@@ -3035,17 +3455,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>COM(2021)769 final Proposal for a DIRECTIVE OF THE EUROPEAN PARLIAMENT AND OF Obsolete - since the adoption of this proposal in 2021, a</t>
+          <t>COM(2011)714 final Proposal for a COUNCIL DIRECTIVE on a common system of taxation Obsolete – the scope of the proposal has been partly</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2021/0400 (COD) THE COUNCIL laying down for certain road vehicles circulating within the recent amendment has been proposed by the Union the maximum authorised dimensions in national and international traffic Commission, that will make this codification proposal and the maximum authorised weights in international traffic (codification) obsolete. The Commission will propose a new codified proposal as soon as the new amendment will have been adopted.</t>
+          <t>2011/0314 (CNS) applicable to interest and royalty payments made between associated companies taken over by the Directive implementing the OECD of different Member States Pillar 2 on minimum corporate taxation. The remaining issues the proposal intended to tackle will be addressed via an upcoming Omnibus act as a part of the simplification process.</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -3056,7 +3476,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2011</t>
         </is>
       </c>
     </row>
@@ -3073,28 +3493,28 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>COM(2022)222 final Proposal for a DIRECTIVE OF THE EUROPEAN PARLIAMENT AND OF Obsolete – the changes suggested by this proposal were</t>
+          <t>COM(2011)827 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF Obsolete – the proposal is by now obsolete. The</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2022/0160 (COD) THE COUNCIL amending Directive (EU) 2018/2001 on the promotion of the incorporated during the discussions on the revision of use of energy from renewable sources, Directive 2010/31/EU on the energy the Energy Performance of Buildings Directive, the performance of buildings and Directive 2012/27/EU on energy efficiency Energy Efficiency Directive and the Renewable Energy Directive.</t>
+          <t>2011/0391 (COD) THE COUNCIL on common rules for the allocation of slots at European Union Commission has launched a fitness-check and will airports decide on the basis of its findings on the way forward.</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>DIRECTIVE</t>
+          <t>REGULATION</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2011</t>
         </is>
       </c>
     </row>
@@ -3111,17 +3531,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>COM(2023)232 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement - the Commission will assess</t>
+          <t>COM(2012)336 final Proposal for a COUNCIL REGULATION establishing a facility for providing Obsolete – the proposal needs to be updated as regards</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>2023/0133(COD) THE COUNCIL on standard essential patents and amending Regulation whether another proposal should be tabled or another (EU)2017/1001 type of approach should be chosen. A new era for European Defence and Security</t>
+          <t>2012/0164 (APP) financial assistance for Member States whose currency is not the euro i.a. the funding modalities of the Balance of Payments Facility and to integrate the lessons to be drawn from the recent crises, as well as the institutional, economic and financial sector developments since 2009, and their possible implication for the design and implementation of the facility, in line with the Council Conclusions of 27 March 2024.</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -3132,7 +3552,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2012</t>
         </is>
       </c>
     </row>
@@ -3149,28 +3569,28 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>COM(2018)634 final Proposal for a DIRECTIVE OF THE EUROPEAN PARLIAMENT AND OF Obsolete - the Commission intends to present a new</t>
+          <t>COM(2015)603 final Proposal for a COUNCIL DECISION laying down measures in view of No foreseeable agreement – in the context of the</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2018/0329 (COD) THE COUNCIL on common standards and procedures in Member States for proposal in 2025 (referred to in annex 1 of this returning illegally staying third-country nationals (recast) A contribution from Commission Work Programme) in the context of which the European Commission to the Leaders’ meeting in Salzburg on 19-20 the current pending proposal will be effectively September 2018 withdrawn.</t>
+          <t>2015/0250 (NLE) progressively establishing unified representation of the euro area in the discussions on Europe’s economic and financial International Monetary Fund sovereignty, the Commission will assess whether another proposal should be tabled or another type of approach should be chosen. 2 This list includes pending legislative proposals, which the Commission intends to withdraw within six months 22 No. References Title Reasons for withdrawal</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>DIRECTIVE</t>
+          <t>DECISION</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2015</t>
         </is>
       </c>
     </row>
@@ -3187,28 +3607,28 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>COM(2021)890 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF Obsolete – the content of this proposal was merged into</t>
+          <t>COM(2017)276 final Proposal for a COUNCIL DIRECTIVE amending Directive 1999/62/EC on the No foreseeable agreement – the proposal is blocked with</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>2021/0427 (COD) THE COUNCIL addressing situations of instrumentalisation in the field of Regulation (EU) 2024/1359 addressing situations of migration and asylum crisis and force majeure in the field of migration and asylum and amending Regulation (EU) 2021/1147.</t>
+          <t>2017/0115 (CNS) charging of heavy goods vehicles for the use of certain infrastructures, as regards no perspective of agreement. certain provisions on vehicle taxation</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>REGULATION</t>
+          <t>DIRECTIVE</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
@@ -3225,28 +3645,28 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>COM(2021)752 final Proposal for a COUNCIL DECISION on provisional emergency measures for Obsolete – the proposal was blocked during the inter-</t>
+          <t>COM(2017)647 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – the proposal has not been</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>2021/0401 (CNS) the benefit of Latvia, Lithuania and Poland institutional discussions and is now obsolete. 24 No. References Title Reasons for withdrawal</t>
+          <t>2017/0288 (COD) THE COUNCIL amending Regulation (EC) No 1073/2009 on common rules for taken up for discussion in the Council and is by now access to the international market for coach and bus services outdated.</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>DECISION</t>
+          <t>REGULATION</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
@@ -3263,28 +3683,28 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>COM(2024)174 final Proposal for a COUNCIL RECOMMENDATION for the 2024/2025 Schengen Obsolete – no agreement was foreseeable. The Schengen</t>
+          <t>COM(2017)827 final Proposal for a COUNCIL REGULATION on the establishment of the European No foreseeable agreement - many of the changes</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2024/0094 (NLE) Cycle Council agreed on a number of priority areas for action that are dealt with via other means than this proposal. Sustaining our quality of life: food security, water and nature</t>
+          <t>2017/0333 (APP) Monetary Fund proposed under this initiative have been incorporated into a separate revision of the European Stability Mechanism Treaty.</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>RECOMMENDATION</t>
+          <t>REGULATION</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
@@ -3301,28 +3721,28 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>COM(2012)403 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected.</t>
+          <t>COM(2018)135 final Proposal for a DIRECTIVE OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – the proposal is blocked and</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>2012/0196 (COD) THE COUNCIL on the protection of species of wild fauna and flora by regulating Furthermore, since 2012, developments took place that trade therein (Recast) make this proposal obsolete. The Commission will assess whether another proposal should be tabled or another type of approach should be chosen to allow for a new start.</t>
+          <t>2018/0063B (COD) THE COUNCIL on credit servicers, credit purchasers and the recovery of further progress is unlikely. collateral</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>REGULATION</t>
+          <t>DIRECTIVE</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
@@ -3339,28 +3759,28 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>COM(2015)177 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement - any potential further</t>
+          <t>COM(2018)329 final Proposal for a COUNCIL DIRECTIVE amending Directive 2006/112/EC as No foreseeable agreement – discussions are suspended</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>2015/0093 (COD) THE COUNCIL amending Regulation (EC) No 1829/2003 as regards the amendment of the GMO legislation will depend on the possibility for the Member States to restrict or prohibit the use of genetically outcome of the negotiations on the proposal for new modified food and feed on their territory genomic techniques, or the identification of issues to be addressed in the context of the biotechnology and biomanufacturing initiative.</t>
+          <t>2018/0164(CNS) regards the introduction of the detailed technical measures for the operation of since 2019 and further progress is unlikely. the definitive VAT system for the taxation of trade between Member States</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>REGULATION</t>
+          <t>DIRECTIVE</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
@@ -3377,17 +3797,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>COM(2022)563 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected</t>
+          <t>COM(2018)339 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – the proposal is blocked and</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2022/0348 (COD) THE COUNCIL laying down management, conservation and control measures between the European Parliament and the Council at applicable in the Area of the Southern Indian Ocean Fisheries Agreement first reading. The Commission intends to present a new (SIOFA) proposal in 2025 in the context of which the current pending proposal will be effectively withdrawn.</t>
+          <t>2018/0171 (COD) THE COUNCIL on sovereign bond-backed securities further progress is unlikely.</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -3398,7 +3818,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
@@ -3415,17 +3835,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>COM(2023)771 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected</t>
+          <t>COM(2018)387 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement - The proposal is outdated</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>2023/0449 (COD) THE COUNCIL amending Regulations (EU) 2016/1139, (EU) 2018/973 and from the colegislators. (EU) 2019/472 as regards the targets for fixing fishing opportunities Protecting our democracy, upholding our values</t>
+          <t>2018/0212 (COD) THE COUNCIL on the establishment of a European Investment Stabilisation with the entry into force of NGEU and the Recovery and Function Resilience Facility (RRF) and the withdrawal of the so- called Budgetary Instrument for Convergence and Competitiveness (BICC) in February 2021.</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -3436,7 +3856,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
@@ -3453,28 +3873,28 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>COM(2008)426 final Proposal for a COUNCIL DIRECTIVE on implementing the principle of equal No foreseeable agreement – the proposal is blocked and</t>
+          <t>COM(2019)38 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF Obsolete – changes contained in this proposal have been</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>2008/0140 (CNS) treatment between persons irrespective of religion or belief, disability, age or further progress is unlikely. sexual orientation 25 No. References Title Reasons for withdrawal</t>
+          <t>2019/0017 (COD) THE COUNCIL amending Regulation (EU) 2015/757 in order to take incorporated into the most recent EU ETS revision, appropriate account of the global data collection system for ship fuel oil adopted in 2023. consumption data</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>DIRECTIVE</t>
+          <t>REGULATION</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>2019</t>
         </is>
       </c>
     </row>
@@ -3491,28 +3911,28 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>COM(2011)137 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND No foreseeable agreement - no progress has been made</t>
+          <t>COM(2020)49 final Proposal for a COUNCIL DIRECTIVE on administrative cooperation in the field Obsolete - since the adoption of this proposal in 2020, a</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>2011/0073 (COD) OF THE COUNCIL amending Regulation (EC) No 1049/2001 regarding public since 2011. access to European Parliament, Council and Commission documents COM(2008)229 final 2008/0090 (COD)</t>
+          <t>2020/0022 (CNS) of taxation (codification) number of significant amendments have been adopted, making this codification proposal obsolete. The Commission will propose a new codified proposal. 23 No. References Title Reasons for withdrawal</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>REGULATION</t>
+          <t>DIRECTIVE</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
@@ -3529,17 +3949,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>COM(2016)799 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND No foreseeable agreement – the proposal is blocked and</t>
+          <t>COM(2020)577 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF Obsolete – changes contained in this proposal have been</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>2016/0400B (COD) OF THE COUNCIL adapting a number of legal acts providing for the use of the further progress is unlikely. There is a legal obligation regulatory procedure with scrutiny to Articles 290 and 291 of the Treaty on the to put legal acts adopted prior to the entry into force of Functioning of the European Union the Treaty of Lisbon in conformity with Articles 290 and 291 TFEU. The Commission will therefore present to the colegislators a new proposal to that effect.</t>
+          <t>2020/0264 (COD) THE COUNCIL amending Regulation (EU) 2018/1139 as regards the capacity incorporated into the Single European Sky ("SES II +") of the European Union Aviation Safety Agency to act as Performance Review Regulation. Body of the Single European Sky</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -3550,7 +3970,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
@@ -3567,28 +3987,28 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>COM(2017)10 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected</t>
+          <t>COM(2021)769 final Proposal for a DIRECTIVE OF THE EUROPEAN PARLIAMENT AND OF Obsolete - since the adoption of this proposal in 2021, a</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2017/0003 (COD) THE COUNCIL concerning the respect for private life and the protection of from the colegislators. Furthermore, the proposal is personal data in electronic communications and repealing Directive 2002/58/EC outdated in view of some recent legislation in both the (Regulation on Privacy and Electronic Communications technological and the legislative landscape.</t>
+          <t>2021/0400 (COD) THE COUNCIL laying down for certain road vehicles circulating within the recent amendment has been proposed by the Union the maximum authorised dimensions in national and international traffic Commission, that will make this codification proposal and the maximum authorised weights in international traffic (codification) obsolete. The Commission will propose a new codified proposal as soon as the new amendment will have been adopted.</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>REGULATION</t>
+          <t>DIRECTIVE</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
@@ -3605,28 +4025,28 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>COM(2017)85 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – the proposal is blocked and</t>
+          <t>COM(2022)222 final Proposal for a DIRECTIVE OF THE EUROPEAN PARLIAMENT AND OF Obsolete – the changes suggested by this proposal were</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>2017/0035 (COD) THE COUNCIL amending Regulation (EU) No 182/2011 laying down the rules further progress is unlikely. and general principles concerning mechanisms for control by Member States of the Commission’s exercise of implementing powers</t>
+          <t>2022/0160 (COD) THE COUNCIL amending Directive (EU) 2018/2001 on the promotion of the incorporated during the discussions on the revision of use of energy from renewable sources, Directive 2010/31/EU on the energy the Energy Performance of Buildings Directive, the performance of buildings and Directive 2012/27/EU on energy efficiency Energy Efficiency Directive and the Renewable Energy Directive.</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>REGULATION</t>
+          <t>DIRECTIVE</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
@@ -3643,17 +4063,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>COM(2018)96 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – the proposal is blocked and</t>
+          <t>COM(2023)232 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement - the Commission will assess</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>2018/0044 (COD) THE COUNCIL on the law applicable to the third-party effects of assignments further progress is unlikely. of claims</t>
+          <t>2023/0133(COD) THE COUNCIL on standard essential patents and amending Regulation whether another proposal should be tabled or another (EU)2017/1001 type of approach should be chosen. A new era for European Defence and Security</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -3664,7 +4084,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
@@ -3681,17 +4101,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>COM(2022)496 final Proposal for a DIRECTIVE OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement - the Commission will assess</t>
+          <t>COM(2018)634 final Proposal for a DIRECTIVE OF THE EUROPEAN PARLIAMENT AND OF Obsolete - the Commission intends to present a new</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>2022/0303 (COD) THE COUNCIL on adapting non-contractual civil liability rules to artificial whether another proposal should be tabled or another intelligence (AI Liability) type of approach should be chosen. A global Europe: Leveraging our power and partnerships</t>
+          <t>2018/0329 (COD) THE COUNCIL on common standards and procedures in Member States for proposal in 2025 (referred to in annex 1 of this returning illegally staying third-country nationals (recast) A contribution from Commission Work Programme) in the context of which the European Commission to the Leaders’ meeting in Salzburg on 19-20 the current pending proposal will be effectively September 2018 withdrawn.</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -3702,7 +4122,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
@@ -3719,28 +4139,28 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>JOIN(2015)36 final Joint Proposal for a COUNCIL DECISION on the conclusion, on behalf of the Obsolete – the ratification process of this agreement has</t>
+          <t>COM(2021)890 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF Obsolete – the content of this proposal was merged into</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2015/0302 (NLE) European Union, of the Cooperation Agreement on Partnership and Development been interrupted with the establishment of a Taliban between the European Union and the Islamic Republic of Afghanistan appointed caretaker government that, to date, remains unrecognized by the international community, making the original agreement obsolete. 26 No. References Title Reasons for withdrawal</t>
+          <t>2021/0427 (COD) THE COUNCIL addressing situations of instrumentalisation in the field of Regulation (EU) 2024/1359 addressing situations of migration and asylum crisis and force majeure in the field of migration and asylum and amending Regulation (EU) 2021/1147.</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>DECISION</t>
+          <t>REGULATION</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
@@ -3757,17 +4177,17 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>COM(2022)63 final Proposal for a COUNCIL DECISION on the position to be taken on behalf of the Obsolete - the proposal was made in the negotiations on</t>
+          <t>COM(2021)752 final Proposal for a COUNCIL DECISION on provisional emergency measures for Obsolete – the proposal was blocked during the inter-</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>2022/0043 (NLE) European Union in the written procedure by the Participants to the Arrangement the modernisation of the Arrangement on Officially on Officially Supported Export Credits amending Annex IV Supported Export Credits, which were finalised in 2023. The content of this proposal was included in another Council decision making this one redundant. Delivering together and preparing our Union for the future</t>
+          <t>2021/0401 (CNS) the benefit of Latvia, Lithuania and Poland institutional discussions and is now obsolete. 24 No. References Title Reasons for withdrawal</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -3778,7 +4198,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
@@ -3795,28 +4215,28 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>COM(2022)184 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF Obsolete - the content of the proposal has been adopted</t>
+          <t>COM(2024)174 final Proposal for a COUNCIL RECOMMENDATION for the 2024/2025 Schengen Obsolete – no agreement was foreseeable. The Schengen</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>2022/0125 (COD) THE COUNCIL amending Regulation (EU, Euratom) 2018/1046 on the financial end of September 2024 as part of the revision of the rules applicable to the general budget of the Union Financial Regulation (Recast).</t>
+          <t>2024/0094 (NLE) Cycle Council agreed on a number of priority areas for action that are dealt with via other means than this proposal. Sustaining our quality of life: food security, water and nature</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>REGULATION</t>
+          <t>RECOMMENDATION</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
@@ -3833,17 +4253,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>COM(2024)301 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected.</t>
+          <t>COM(2012)403 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected.</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>2024/0059 (COD) THE COUNCIL amending Regulation (EU) 2021/1148 as regards the financial Furthermore, the MFF mid-term revision can be envelope and the allocation for the thematic facility implemented without this legal proposal.</t>
+          <t>2012/0196 (COD) THE COUNCIL on the protection of species of wild fauna and flora by regulating Furthermore, since 2012, developments took place that trade therein (Recast) make this proposal obsolete. The Commission will assess whether another proposal should be tabled or another type of approach should be chosen to allow for a new start.</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -3854,7 +4274,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2012</t>
         </is>
       </c>
     </row>
@@ -3871,17 +4291,17 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>23</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>COM(2024)100 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected.</t>
+          <t>COM(2015)177 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement - any potential further</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>2024/0060 (COD) THE COUNCIL amending Regulation (EU) No 2021/522, Regulation (EU) No The MFF mid-term revision can be implemented 2021/1057, Regulation (EU) No 2021/1060, Regulation (EU) No 2021/1139, without this legal proposal. An amendment to the Regulation (EU) No 2021/1229 and Regulation (EU) No 2021/1775 as regards Regulation 2021/1755 establishing the Brexit the changes to the amounts of funds for certain programmes and funds Adjustment Reserve (BAR) to establish the legal basis for redistribution of the outstanding amounts between the Member States will be proposed by the Commission in 2025. 27 Annex V: Envisaged repeals No. Policy area Title Reasons for repeal</t>
+          <t>2015/0093 (COD) THE COUNCIL amending Regulation (EC) No 1829/2003 as regards the amendment of the GMO legislation will depend on the possibility for the Member States to restrict or prohibit the use of genetically outcome of the negotiations on the proposal for new modified food and feed on their territory genomic techniques, or the identification of issues to be addressed in the context of the biotechnology and biomanufacturing initiative.</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -3892,7 +4312,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2015</t>
         </is>
       </c>
     </row>
@@ -3909,28 +4329,28 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Agriculture Council Regulation (EC)No 870/2004 of 26 This Community programme was established for the period 2004 to 2006 to complement and</t>
+          <t>COM(2022)563 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>April 2004 establishing a Community promote, at Community level, the work undertaken in the Member States for the conservation, programme on the conservation, characterisation, collection and utilisation of genetic resources in agriculture. Support under this characterisation, collection and utilisation of programme is no longer available, since all Common Agricultural Policy (CAP) support is currently genetic resources in agriculture and repealing granted under the ongoing rural development programmes (until 2025) and national CAP Strategic Regulation (EC) No 1467/94 Plans (until 2027), following Regulation (EU) 1305/2013 and Regulation (EU) 2021/2115 respectively, making this regulation obsolete.</t>
+          <t>2022/0348 (COD) THE COUNCIL laying down management, conservation and control measures between the European Parliament and the Council at applicable in the Area of the Southern Indian Ocean Fisheries Agreement first reading. The Commission intends to present a new (SIOFA) proposal in 2025 in the context of which the current pending proposal will be effectively withdrawn.</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Regulation</t>
+          <t>REGULATION</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
@@ -3947,28 +4367,28 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>European statistics Council Regulation (EEC) No 3037/90 of 9 The classification from 1990 is obsolete. The current statistical classification of economic</t>
+          <t>COM(2023)771 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>October 1990 on the statistical classification of activities’ in the European Community (NACE) is established in Regulation (EC) No 1893/2006 economic activities in the European of the European Parliament and of the Council of 20 December 2006, as last amended by Community Commission Delegated Regulation (EU) 2023/137 of 10 October 2022.</t>
+          <t>2023/0449 (COD) THE COUNCIL amending Regulations (EU) 2016/1139, (EU) 2018/973 and from the colegislators. (EU) 2019/472 as regards the targets for fixing fishing opportunities Protecting our democracy, upholding our values</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Regulation</t>
+          <t>REGULATION</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>2006</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
@@ -3985,26 +4405,30 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>European statistics Council Decision of 25 June 1996 on improving The Decision is obsolete. It has been superseded by new regulations on agricultural statistics</t>
+          <t>COM(2008)426 final Proposal for a COUNCIL DIRECTIVE on implementing the principle of equal No foreseeable agreement – the proposal is blocked and</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Community agricultural statistics (96/411/EC) (integrated farm statistics, agricultural input and output, economic accounts for agriculture).</t>
+          <t>2008/0140 (CNS) treatment between persons irrespective of religion or belief, disability, age or further progress is unlikely. sexual orientation 25 No. References Title Reasons for withdrawal</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="H113" t="inlineStr"/>
+          <t>DIRECTIVE</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4019,26 +4443,554 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Road freight Council Regulation (EEC) No 4058/89 of 21 Modern EU legislation has introduced a comprehensive framework that regulates road transport,</t>
+          <t>COM(2011)137 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND No foreseeable agreement - no progress has been made</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>transport December 1989 on the fixing of rates for the focusing on safety, environmental standards, and fair competition without the need for rate-fixing. carriage of goods by road between Member Regulations such as Regulation (EC) No 1071/2009, Regulation (EC) No 1072/2009, and States Regulation (EC) No 1073/2009 have effectively superseded the need for the provisions outlined in Council Regulation (EEC) No 4058/89, rendering it redundant. 28</t>
+          <t>2011/0073 (COD) OF THE COUNCIL amending Regulation (EC) No 1049/2001 regarding public since 2011. access to European Parliament, Council and Commission documents COM(2008)229 final 2008/0090 (COD)</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Regulation</t>
+          <t>REGULATION</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>WP114</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>COM(2016)799 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND No foreseeable agreement – the proposal is blocked and</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>2016/0400B (COD) OF THE COUNCIL adapting a number of legal acts providing for the use of the further progress is unlikely. There is a legal obligation regulatory procedure with scrutiny to Articles 290 and 291 of the Treaty on the to put legal acts adopted prior to the entry into force of Functioning of the European Union the Treaty of Lisbon in conformity with Articles 290 and 291 TFEU. The Commission will therefore present to the colegislators a new proposal to that effect.</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>REGULATION</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>WP115</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>COM(2017)10 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>2017/0003 (COD) THE COUNCIL concerning the respect for private life and the protection of from the colegislators. Furthermore, the proposal is personal data in electronic communications and repealing Directive 2002/58/EC outdated in view of some recent legislation in both the (Regulation on Privacy and Electronic Communications technological and the legislative landscape.</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>REGULATION</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>WP116</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>COM(2017)85 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – the proposal is blocked and</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>2017/0035 (COD) THE COUNCIL amending Regulation (EU) No 182/2011 laying down the rules further progress is unlikely. and general principles concerning mechanisms for control by Member States of the Commission’s exercise of implementing powers</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>REGULATION</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>WP117</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>COM(2018)96 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – the proposal is blocked and</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>2018/0044 (COD) THE COUNCIL on the law applicable to the third-party effects of assignments further progress is unlikely. of claims</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>REGULATION</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>WP118</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>COM(2022)496 final Proposal for a DIRECTIVE OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement - the Commission will assess</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>2022/0303 (COD) THE COUNCIL on adapting non-contractual civil liability rules to artificial whether another proposal should be tabled or another intelligence (AI Liability) type of approach should be chosen. A global Europe: Leveraging our power and partnerships</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>DIRECTIVE</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>WP119</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>JOIN(2015)36 final Joint Proposal for a COUNCIL DECISION on the conclusion, on behalf of the Obsolete – the ratification process of this agreement has</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2015/0302 (NLE) European Union, of the Cooperation Agreement on Partnership and Development been interrupted with the establishment of a Taliban between the European Union and the Islamic Republic of Afghanistan appointed caretaker government that, to date, remains unrecognized by the international community, making the original agreement obsolete. 26 No. References Title Reasons for withdrawal</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>DECISION</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>WP120</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>COM(2022)63 final Proposal for a COUNCIL DECISION on the position to be taken on behalf of the Obsolete - the proposal was made in the negotiations on</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2022/0043 (NLE) European Union in the written procedure by the Participants to the Arrangement the modernisation of the Arrangement on Officially on Officially Supported Export Credits amending Annex IV Supported Export Credits, which were finalised in 2023. The content of this proposal was included in another Council decision making this one redundant. Delivering together and preparing our Union for the future</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>DECISION</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>WP121</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>COM(2022)184 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF Obsolete - the content of the proposal has been adopted</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2022/0125 (COD) THE COUNCIL amending Regulation (EU, Euratom) 2018/1046 on the financial end of September 2024 as part of the revision of the rules applicable to the general budget of the Union Financial Regulation (Recast).</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>REGULATION</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>WP122</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>COM(2024)301 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected.</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2024/0059 (COD) THE COUNCIL amending Regulation (EU) 2021/1148 as regards the financial Furthermore, the MFF mid-term revision can be envelope and the allocation for the thematic facility implemented without this legal proposal.</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>REGULATION</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>WP123</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>COM(2024)100 final Proposal for a REGULATION OF THE EUROPEAN PARLIAMENT AND OF No foreseeable agreement – no agreement is expected.</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2024/0060 (COD) THE COUNCIL amending Regulation (EU) No 2021/522, Regulation (EU) No The MFF mid-term revision can be implemented 2021/1057, Regulation (EU) No 2021/1060, Regulation (EU) No 2021/1139, without this legal proposal. An amendment to the Regulation (EU) No 2021/1229 and Regulation (EU) No 2021/1775 as regards Regulation 2021/1755 establishing the Brexit the changes to the amounts of funds for certain programmes and funds Adjustment Reserve (BAR) to establish the legal basis for redistribution of the outstanding amounts between the Member States will be proposed by the Commission in 2025. 27 Annex V: Envisaged repeals No. Policy area Title Reasons for repeal</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>REGULATION</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>WP124</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Agriculture Council Regulation (EC)No 870/2004 of 26 This Community programme was established for the period 2004 to 2006 to complement and</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>April 2004 establishing a Community promote, at Community level, the work undertaken in the Member States for the conservation, programme on the conservation, characterisation, collection and utilisation of genetic resources in agriculture. Support under this characterisation, collection and utilisation of programme is no longer available, since all Common Agricultural Policy (CAP) support is currently genetic resources in agriculture and repealing granted under the ongoing rural development programmes (until 2025) and national CAP Strategic Regulation (EC) No 1467/94 Plans (until 2027), following Regulation (EU) 1305/2013 and Regulation (EU) 2021/2115 respectively, making this regulation obsolete.</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>REGULATION</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>WP125</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>European statistics Council Regulation (EEC) No 3037/90 of 9 The classification from 1990 is obsolete. The current statistical classification of economic</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>October 1990 on the statistical classification of activities’ in the European Community (NACE) is established in Regulation (EC) No 1893/2006 economic activities in the European of the European Parliament and of the Council of 20 December 2006, as last amended by Community Commission Delegated Regulation (EU) 2023/137 of 10 October 2022.</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>REGULATION</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>WP126</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>European statistics Council Decision of 25 June 1996 on improving The Decision is obsolete. It has been superseded by new regulations on agricultural statistics</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Community agricultural statistics (96/411/EC) (integrated farm statistics, agricultural input and output, economic accounts for agriculture).</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>DECISION</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>WP127</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Road freight Council Regulation (EEC) No 4058/89 of 21 Modern EU legislation has introduced a comprehensive framework that regulates road transport,</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>transport December 1989 on the fixing of rates for the focusing on safety, environmental standards, and fair competition without the need for rate-fixing. carriage of goods by road between Member Regulations such as Regulation (EC) No 1071/2009, Regulation (EC) No 1072/2009, and States Regulation (EC) No 1073/2009 have effectively superseded the need for the provisions outlined in Council Regulation (EEC) No 4058/89, rendering it redundant. 28</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>REGULATION</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
         <is>
           <t>2009</t>
         </is>

</xml_diff>